<commit_message>
Replace Excel plan with updated version
</commit_message>
<xml_diff>
--- a/TS presentation 270526/taelskridt-plan-dk.xlsx
+++ b/TS presentation 270526/taelskridt-plan-dk.xlsx
@@ -1,18 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\coman\Desktop\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84CDD643-79DE-466C-8861-70DFF33610BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-16920" yWindow="-16320" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Generelt" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="UX" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Marketing" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Generelt" sheetId="1" r:id="rId1"/>
+    <sheet name="UX" sheetId="2" r:id="rId2"/>
+    <sheet name="Marketing" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -24,1019 +29,1016 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="305">
   <si>
-    <t xml:space="preserve">Tæl Skridt — Plan frem mod TS3 2026 (Tæl Skridt For Hjertet)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Planperiode: 1. juni 2026 — 13. september 2026 | Kampagne: 31. aug – 13. sep 2026 | Partnerskab: Hjerteforeningen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mål: fastholde tidligere holdkaptajner og deres hold; rekruttere nye arbejdspladser og deltagere</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase-oversigt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase 1: Fundament (1.–28. juni)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking, UTM-oprydning, evergreen-indhold, listebygning, LinkedIn-test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase 2: Optakt inkl. sommer (29. juni – 9. aug)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Før-sommer-push, sommerpause, kreativ produktion, Hjerteforeningen-annoncering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase 3: Lancering (10. – 30. aug)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aktiv rekruttering. Betalt Meta, betalt Google, e-mail, LinkedIn skaleret</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase 4: Kampagnen kører (31. aug – 13. sep)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fastholdelse, motivation, daglig engagement. Fra rekruttering til service</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase 5: Efter kampagnen (14.–20. sep)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retrospektiv, læringer, takke-kommunikation, forberedelse til TS4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marketingbudget</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Post</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bemærkninger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LinkedIn-test (SammenholdsID, B2B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.000 kr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4-ugers test i juni. Læringsspend.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betalt Meta (lanceringsvindue)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12.000 kr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vægtet man–tirs, 06:00–13:00 og 19:00–21:00.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betalt Google Search</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.000 kr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brandede + kategori-relaterede søgeord.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LinkedIn skalering (hvis testen virker)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.000 kr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reserve til august-push, hvis juni-testen leverer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kreativ produktion (foto/video)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.000 kr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lifestyle-fotografi eller stock-licens.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I alt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">30.000 kr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inden for budgetrammen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Succeskriterier for TS3 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Måling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hvad det måler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sådan måles det</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fastholdelsesrate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% af tidligere holdkaptajner der genaktiverer deres hold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sammenkøres fra tidligere kampagnelister og TS3-tilmeldinger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nye arbejdspladser</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Antal nye arbejdspladser tilmeldt TS3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Førstegangs-SammenholdsID og enkeltstående hold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nyhedsbrev-tilvækst</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Samlet antal abonnenter pr. 30. august</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mål: +1.500 i forhold til nuværende baseline gennem fase 1+2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LinkedIn-test resultat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pris pr. SammenholdsID-relevant klik og evt. tilmeldinger</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grundlag for beslutning om august-skalering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail åbnings- og klikrater</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Åbning og klik på fastholdelses-e-mails til tidligere deltagere</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Især 'kom tilbage'-sekvensen i fase 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking-klarhed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clarity aktiv, smart events virker, baseline-data fanget</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Binær: ja/nej inden midten af august</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ugentligt overblik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Datoer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UX-fokus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marketing-fokus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Milepæle / leverancer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 jun – 7 jun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fundament</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Geninstaller Clarity på site + platform; opsæt smart events</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indfør nye UTM-konventioner på alle kanaler; brief LinkedIn-test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clarity aktiv på begge flader inden fredag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8 jun – 14 jun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Påbegynd redesign af forsidens øverste del; audit af OG-preview</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lancér LinkedIn SammenholdsID-test (4 uger); første Walk of Fame-historie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LinkedIn live; OG-preview forbedret</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">15 jun – 21 jun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fortsæt redesign; træk Clarity-optagelser fra step-input-side</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Push for nyhedsbrev-tilmelding på forsiden; anden Walk of Fame-historie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Audit-dokument for step-input-siden klar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22 jun – 28 jun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lancér forsidens nye øverste del</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail til tidligere holdkaptajner: 'Tæl Skridt For Hjertet starter 31. august'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forside v2 live; første fastholdelses-e-mail sendt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29 jun – 5 jul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Definér rettelser til step-input-siden; audit af profilside</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annoncering af Hjerteforeningen-partnerskab (organisk + e-mail)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hjerteforeningen-partnerskab offentliggjort</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 jul – 12 jul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Optakt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sidste arbejdsuge før sommer; brief TS3-kreativ produktion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Soft e-mail til tidligere deltagere: 'kom tilbage – nu med Hjerteforeningen'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS3 kreativt brief leveret</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13 jul – 19 jul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sommerpause — kun vedligehold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sommerpause for betalt; organisk holder tempo med Benspænd-indhold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">20 jul – 26 jul</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sommerpause fortsætter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">27 jul – 2 aug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sommerpause; LinkedIn-resultater gennemgået</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LinkedIn fase 1-resultater; beslutning om skalering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LinkedIn-beslutning dokumenteret</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 32</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 aug – 9 aug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modtag TS3 kreativ; sidste platform-QA på Edge + iOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail varme-op-sekvens til tidligere deltagere starter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alle kreative leverancer modtaget og godkendt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 33</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10 aug – 16 aug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lancering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sidste test før lancering; freeze-øvelse for site + platform</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betalt Meta + Google lanceres; 'sidste chance for tilmelding'-flow live</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betalte kampagner live mandag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 34</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17 aug – 23 aug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Endelig freeze; QA-runde identisk med launch-dag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail til hele listen: TS3 starter på mandag; LinkedIn skalering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Site og platform frosset inden fredag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 aug – 30 aug</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Daglig Clarity-overvågning; smart events gennemgang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kickoff-opslag; daglige lykkehjul-vindere på social</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS3 LIVE — 31. august kl. 00:01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31 aug – 6 sep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kampagnen kører</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Midt-kampagne engagement-push; bug-triage på platform</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Midt-kampagne motivations-e-mail; nudge til lav-aktive holdkaptajner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Midt-kampagne tjek-ind</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7 sep – 13 sep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slut-overvågning; indsaml Walk of Fame-historier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sidste-dage-push e-mail; tak-opslag på social</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS3 slutter søndag 13. september</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uge 38</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14 sep – 20 sep</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Efter kampagnen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Efter-kampagne retrospektiv; dokumentér læringer til TS4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tak-e-mail til alle deltagere; Walk of Fame-historier samlet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retrospektiv-dokument klar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UX-plan — én designer, 14 uger frem mod TS3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Realistisk kapacitet: 2-3 timer pr. dag på TS, prioriteret efter løftestang.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tema</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opgaver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leverancer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tracking-uge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Geninstaller Clarity-script på taelskridt.dk
+    <t>Tæl Skridt — Plan frem mod TS3 2026 (Tæl Skridt For Hjertet)</t>
+  </si>
+  <si>
+    <t>Planperiode: 1. juni 2026 — 13. september 2026 | Kampagne: 31. aug – 13. sep 2026 | Partnerskab: Hjerteforeningen</t>
+  </si>
+  <si>
+    <t>Mål: fastholde tidligere holdkaptajner og deres hold; rekruttere nye arbejdspladser og deltagere</t>
+  </si>
+  <si>
+    <t>Fase-oversigt</t>
+  </si>
+  <si>
+    <t>Fase 1: Fundament (1.–28. juni)</t>
+  </si>
+  <si>
+    <t>Tracking, UTM-oprydning, evergreen-indhold, listebygning, LinkedIn-test</t>
+  </si>
+  <si>
+    <t>Fase 2: Optakt inkl. sommer (29. juni – 9. aug)</t>
+  </si>
+  <si>
+    <t>Før-sommer-push, sommerpause, kreativ produktion, Hjerteforeningen-annoncering</t>
+  </si>
+  <si>
+    <t>Fase 3: Lancering (10. – 30. aug)</t>
+  </si>
+  <si>
+    <t>Aktiv rekruttering. Betalt Meta, betalt Google, e-mail, LinkedIn skaleret</t>
+  </si>
+  <si>
+    <t>Fase 4: Kampagnen kører (31. aug – 13. sep)</t>
+  </si>
+  <si>
+    <t>Fastholdelse, motivation, daglig engagement. Fra rekruttering til service</t>
+  </si>
+  <si>
+    <t>Fase 5: Efter kampagnen (14.–20. sep)</t>
+  </si>
+  <si>
+    <t>Retrospektiv, læringer, takke-kommunikation, forberedelse til TS4</t>
+  </si>
+  <si>
+    <t>Marketingbudget</t>
+  </si>
+  <si>
+    <t>Post</t>
+  </si>
+  <si>
+    <t>Estimat</t>
+  </si>
+  <si>
+    <t>Bemærkninger</t>
+  </si>
+  <si>
+    <t>LinkedIn-test (SammenholdsID, B2B)</t>
+  </si>
+  <si>
+    <t>7.000 kr</t>
+  </si>
+  <si>
+    <t>4-ugers test i juni. Læringsspend.</t>
+  </si>
+  <si>
+    <t>Betalt Meta (lanceringsvindue)</t>
+  </si>
+  <si>
+    <t>12.000 kr</t>
+  </si>
+  <si>
+    <t>Vægtet man–tirs, 06:00–13:00 og 19:00–21:00.</t>
+  </si>
+  <si>
+    <t>Betalt Google Search</t>
+  </si>
+  <si>
+    <t>6.000 kr</t>
+  </si>
+  <si>
+    <t>Brandede + kategori-relaterede søgeord.</t>
+  </si>
+  <si>
+    <t>LinkedIn skalering (hvis testen virker)</t>
+  </si>
+  <si>
+    <t>3.000 kr</t>
+  </si>
+  <si>
+    <t>Reserve til august-push, hvis juni-testen leverer.</t>
+  </si>
+  <si>
+    <t>Kreativ produktion (foto/video)</t>
+  </si>
+  <si>
+    <t>2.000 kr</t>
+  </si>
+  <si>
+    <t>Lifestyle-fotografi eller stock-licens.</t>
+  </si>
+  <si>
+    <t>I alt</t>
+  </si>
+  <si>
+    <t>30.000 kr</t>
+  </si>
+  <si>
+    <t>Inden for budgetrammen.</t>
+  </si>
+  <si>
+    <t>Succeskriterier for TS3 2026</t>
+  </si>
+  <si>
+    <t>Måling</t>
+  </si>
+  <si>
+    <t>Hvad det måler</t>
+  </si>
+  <si>
+    <t>Sådan måles det</t>
+  </si>
+  <si>
+    <t>Fastholdelsesrate</t>
+  </si>
+  <si>
+    <t>% af tidligere holdkaptajner der genaktiverer deres hold</t>
+  </si>
+  <si>
+    <t>Sammenkøres fra tidligere kampagnelister og TS3-tilmeldinger</t>
+  </si>
+  <si>
+    <t>Nye arbejdspladser</t>
+  </si>
+  <si>
+    <t>Antal nye arbejdspladser tilmeldt TS3</t>
+  </si>
+  <si>
+    <t>Førstegangs-SammenholdsID og enkeltstående hold</t>
+  </si>
+  <si>
+    <t>Nyhedsbrev-tilvækst</t>
+  </si>
+  <si>
+    <t>Samlet antal abonnenter pr. 30. august</t>
+  </si>
+  <si>
+    <t>Mål: +1.500 i forhold til nuværende baseline gennem fase 1+2</t>
+  </si>
+  <si>
+    <t>LinkedIn-test resultat</t>
+  </si>
+  <si>
+    <t>Pris pr. SammenholdsID-relevant klik og evt. tilmeldinger</t>
+  </si>
+  <si>
+    <t>Grundlag for beslutning om august-skalering</t>
+  </si>
+  <si>
+    <t>E-mail åbnings- og klikrater</t>
+  </si>
+  <si>
+    <t>Åbning og klik på fastholdelses-e-mails til tidligere deltagere</t>
+  </si>
+  <si>
+    <t>Især 'kom tilbage'-sekvensen i fase 2</t>
+  </si>
+  <si>
+    <t>Tracking-klarhed</t>
+  </si>
+  <si>
+    <t>Clarity aktiv, smart events virker, baseline-data fanget</t>
+  </si>
+  <si>
+    <t>Binær: ja/nej inden midten af august</t>
+  </si>
+  <si>
+    <t>Ugentligt overblik</t>
+  </si>
+  <si>
+    <t>Uge</t>
+  </si>
+  <si>
+    <t>Datoer</t>
+  </si>
+  <si>
+    <t>Fase</t>
+  </si>
+  <si>
+    <t>UX-fokus</t>
+  </si>
+  <si>
+    <t>Marketing-fokus</t>
+  </si>
+  <si>
+    <t>Milepæle / leverancer</t>
+  </si>
+  <si>
+    <t>Uge 23</t>
+  </si>
+  <si>
+    <t>1 jun – 7 jun</t>
+  </si>
+  <si>
+    <t>Fundament</t>
+  </si>
+  <si>
+    <t>Geninstaller Clarity på site + platform; opsæt smart events</t>
+  </si>
+  <si>
+    <t>Indfør nye UTM-konventioner på alle kanaler; brief LinkedIn-test</t>
+  </si>
+  <si>
+    <t>Clarity aktiv på begge flader inden fredag</t>
+  </si>
+  <si>
+    <t>Uge 24</t>
+  </si>
+  <si>
+    <t>8 jun – 14 jun</t>
+  </si>
+  <si>
+    <t>Påbegynd redesign af forsidens øverste del; audit af OG-preview</t>
+  </si>
+  <si>
+    <t>Lancér LinkedIn SammenholdsID-test (4 uger); første Walk of Fame-historie</t>
+  </si>
+  <si>
+    <t>LinkedIn live; OG-preview forbedret</t>
+  </si>
+  <si>
+    <t>Uge 25</t>
+  </si>
+  <si>
+    <t>15 jun – 21 jun</t>
+  </si>
+  <si>
+    <t>Fortsæt redesign; træk Clarity-optagelser fra step-input-side</t>
+  </si>
+  <si>
+    <t>Push for nyhedsbrev-tilmelding på forsiden; anden Walk of Fame-historie</t>
+  </si>
+  <si>
+    <t>Audit-dokument for step-input-siden klar</t>
+  </si>
+  <si>
+    <t>Uge 26</t>
+  </si>
+  <si>
+    <t>22 jun – 28 jun</t>
+  </si>
+  <si>
+    <t>Lancér forsidens nye øverste del</t>
+  </si>
+  <si>
+    <t>E-mail til tidligere holdkaptajner: 'Tæl Skridt For Hjertet starter 31. august'</t>
+  </si>
+  <si>
+    <t>Forside v2 live; første fastholdelses-e-mail sendt</t>
+  </si>
+  <si>
+    <t>Uge 27</t>
+  </si>
+  <si>
+    <t>29 jun – 5 jul</t>
+  </si>
+  <si>
+    <t>Definér rettelser til step-input-siden; audit af profilside</t>
+  </si>
+  <si>
+    <t>Annoncering af Hjerteforeningen-partnerskab (organisk + e-mail)</t>
+  </si>
+  <si>
+    <t>Hjerteforeningen-partnerskab offentliggjort</t>
+  </si>
+  <si>
+    <t>Uge 28</t>
+  </si>
+  <si>
+    <t>6 jul – 12 jul</t>
+  </si>
+  <si>
+    <t>Optakt</t>
+  </si>
+  <si>
+    <t>Sidste arbejdsuge før sommer; brief TS3-kreativ produktion</t>
+  </si>
+  <si>
+    <t>Soft e-mail til tidligere deltagere: 'kom tilbage – nu med Hjerteforeningen'</t>
+  </si>
+  <si>
+    <t>TS3 kreativt brief leveret</t>
+  </si>
+  <si>
+    <t>Uge 29</t>
+  </si>
+  <si>
+    <t>13 jul – 19 jul</t>
+  </si>
+  <si>
+    <t>Sommerpause — kun vedligehold</t>
+  </si>
+  <si>
+    <t>Sommerpause for betalt; organisk holder tempo med Benspænd-indhold</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Uge 30</t>
+  </si>
+  <si>
+    <t>20 jul – 26 jul</t>
+  </si>
+  <si>
+    <t>Sommerpause fortsætter</t>
+  </si>
+  <si>
+    <t>Uge 31</t>
+  </si>
+  <si>
+    <t>27 jul – 2 aug</t>
+  </si>
+  <si>
+    <t>Sommerpause; LinkedIn-resultater gennemgået</t>
+  </si>
+  <si>
+    <t>LinkedIn fase 1-resultater; beslutning om skalering</t>
+  </si>
+  <si>
+    <t>LinkedIn-beslutning dokumenteret</t>
+  </si>
+  <si>
+    <t>Uge 32</t>
+  </si>
+  <si>
+    <t>3 aug – 9 aug</t>
+  </si>
+  <si>
+    <t>Modtag TS3 kreativ; sidste platform-QA på Edge + iOS</t>
+  </si>
+  <si>
+    <t>E-mail varme-op-sekvens til tidligere deltagere starter</t>
+  </si>
+  <si>
+    <t>Alle kreative leverancer modtaget og godkendt</t>
+  </si>
+  <si>
+    <t>Uge 33</t>
+  </si>
+  <si>
+    <t>10 aug – 16 aug</t>
+  </si>
+  <si>
+    <t>Lancering</t>
+  </si>
+  <si>
+    <t>Sidste test før lancering; freeze-øvelse for site + platform</t>
+  </si>
+  <si>
+    <t>Betalt Meta + Google lanceres; 'sidste chance for tilmelding'-flow live</t>
+  </si>
+  <si>
+    <t>Betalte kampagner live mandag</t>
+  </si>
+  <si>
+    <t>Uge 34</t>
+  </si>
+  <si>
+    <t>17 aug – 23 aug</t>
+  </si>
+  <si>
+    <t>Endelig freeze; QA-runde identisk med launch-dag</t>
+  </si>
+  <si>
+    <t>E-mail til hele listen: TS3 starter på mandag; LinkedIn skalering</t>
+  </si>
+  <si>
+    <t>Site og platform frosset inden fredag</t>
+  </si>
+  <si>
+    <t>Uge 35</t>
+  </si>
+  <si>
+    <t>24 aug – 30 aug</t>
+  </si>
+  <si>
+    <t>Daglig Clarity-overvågning; smart events gennemgang</t>
+  </si>
+  <si>
+    <t>Kickoff-opslag; daglige lykkehjul-vindere på social</t>
+  </si>
+  <si>
+    <t>TS3 LIVE — 31. august kl. 00:01</t>
+  </si>
+  <si>
+    <t>Uge 36</t>
+  </si>
+  <si>
+    <t>31 aug – 6 sep</t>
+  </si>
+  <si>
+    <t>Kampagnen kører</t>
+  </si>
+  <si>
+    <t>Midt-kampagne engagement-push; bug-triage på platform</t>
+  </si>
+  <si>
+    <t>Midt-kampagne motivations-e-mail; nudge til lav-aktive holdkaptajner</t>
+  </si>
+  <si>
+    <t>Midt-kampagne tjek-ind</t>
+  </si>
+  <si>
+    <t>Uge 37</t>
+  </si>
+  <si>
+    <t>7 sep – 13 sep</t>
+  </si>
+  <si>
+    <t>Slut-overvågning; indsaml Walk of Fame-historier</t>
+  </si>
+  <si>
+    <t>Sidste-dage-push e-mail; tak-opslag på social</t>
+  </si>
+  <si>
+    <t>TS3 slutter søndag 13. september</t>
+  </si>
+  <si>
+    <t>Uge 38</t>
+  </si>
+  <si>
+    <t>14 sep – 20 sep</t>
+  </si>
+  <si>
+    <t>Efter kampagnen</t>
+  </si>
+  <si>
+    <t>Efter-kampagne retrospektiv; dokumentér læringer til TS4</t>
+  </si>
+  <si>
+    <t>Tak-e-mail til alle deltagere; Walk of Fame-historier samlet</t>
+  </si>
+  <si>
+    <t>Retrospektiv-dokument klar</t>
+  </si>
+  <si>
+    <t>UX-plan — én designer, 14 uger frem mod TS3</t>
+  </si>
+  <si>
+    <t>Realistisk kapacitet: 2-3 timer pr. dag på TS, prioriteret efter løftestang.</t>
+  </si>
+  <si>
+    <t>Tema</t>
+  </si>
+  <si>
+    <t>Opgaver</t>
+  </si>
+  <si>
+    <t>Leverancer</t>
+  </si>
+  <si>
+    <t>Noter</t>
+  </si>
+  <si>
+    <t>Tracking-uge</t>
+  </si>
+  <si>
+    <t>• Geninstaller Clarity-script på taelskridt.dk
 • Geninstaller Clarity-script på app.taelskridt.dk
 • Definér smart events sammen med IT Heroes: tilmelding gennemført, første skridt-indtastning, holdkaptajn-invitation sendt, SammenholdsID-dashboard besøgt, lykkehjul-spin
 • Verificér at events fyres på staging + produktion</t>
   </si>
   <si>
-    <t xml:space="preserve">Begge Clarity-scripts live; smart events specifikation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Koordinér tidligt på ugen med IT Heroes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forside-redesign start + OG-audit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Påbegynd redesign af forsidens øverste del: synlig kampagne-nedtælling, ligestil Vær med vs LOG IND visuelt, fremhæv SammenholdsID, løft social proof op over folden
+    <t>Begge Clarity-scripts live; smart events specifikation</t>
+  </si>
+  <si>
+    <t>Koordinér tidligt på ugen med IT Heroes.</t>
+  </si>
+  <si>
+    <t>Forside-redesign start + OG-audit</t>
+  </si>
+  <si>
+    <t>• Påbegynd redesign af forsidens øverste del: synlig kampagne-nedtælling, ligestil Vær med vs LOG IND visuelt, fremhæv SammenholdsID, løft social proof op over folden
 • Audit af Open Graph-preview-kort til Teams/SharePoint/PowerApps deling
 • Ret OG-billede, titel, beskrivelse hvor nødvendigt</t>
   </si>
   <si>
-    <t xml:space="preserve">Forside-mockups (mobil + desktop); OG-preview før/efter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OG-rettelser er en gratis distributionsgevinst.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Step-input-optagelser + iteration</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Træk 20-30 Clarity-optagelser fra step-input-siden, både desktop og mobil
+    <t>Forside-mockups (mobil + desktop); OG-preview før/efter</t>
+  </si>
+  <si>
+    <t>OG-rettelser er en gratis distributionsgevinst.</t>
+  </si>
+  <si>
+    <t>Step-input-optagelser + iteration</t>
+  </si>
+  <si>
+    <t>• Træk 20-30 Clarity-optagelser fra step-input-siden, både desktop og mobil
 • Kategorisér dead-click-mønstre: deaktiveret knap, ser klikbart ud men er ikke, asynkront uden feedback, mobile tap-mål
 • Skriv resultater op
 • Iterér forside-redesign baseret på dev-feedback</t>
   </si>
   <si>
-    <t xml:space="preserve">Audit-dokument for step-input; forside-redesign v2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hvis optagelser viser JS-fejl der blokerer indsendelse, eskalér til IT Heroes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lancér forside; audit af profilside</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Overdrag forside-redesign til IT Heroes til produktions-deploy
+    <t>Audit-dokument for step-input; forside-redesign v2</t>
+  </si>
+  <si>
+    <t>Hvis optagelser viser JS-fejl der blokerer indsendelse, eskalér til IT Heroes.</t>
+  </si>
+  <si>
+    <t>Lancér forside; audit af profilside</t>
+  </si>
+  <si>
+    <t>• Overdrag forside-redesign til IT Heroes til produktions-deploy
 • Audit af /users/edit-siden: træk optagelser, identificér årsag til 45% quickback-rate
 • Skitsér forbedringer til profilsiden</t>
   </si>
   <si>
-    <t xml:space="preserve">Forside v2 live; profilside-resultater</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slut på fase 1. Status før sommer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Step-input-rettelser design + FAQ-promotion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Design af step-input-rettelser baseret på uge 3-resultater — knaptilstande, tap-mål, feedback-tilstande
+    <t>Forside v2 live; profilside-resultater</t>
+  </si>
+  <si>
+    <t>Slut på fase 1. Status før sommer.</t>
+  </si>
+  <si>
+    <t>Step-input-rettelser design + FAQ-promotion</t>
+  </si>
+  <si>
+    <t>• Design af step-input-rettelser baseret på uge 3-resultater — knaptilstande, tap-mål, feedback-tilstande
 • Fremhæv FAQ verifikation + ikke-gå-sport-spørgsmål over folden eller i tilmeldingsflow
 • Overdrag til IT Heroes til bygning (lanceres efter sommer)</t>
   </si>
   <si>
-    <t xml:space="preserve">Step-input-rettelser specifikation; FAQ-promotion-design</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sidste fulde arbejdsuge før sommer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS3 kreativt brief + sommer-forberedelse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Brief TS3 kreativ til fotograf/freelance designer: lifestyle-billeder, kvinder 50+ i danske arbejds- og hjemmekontekster, vertikale mobil-først-formater, Hjerteforeningen co-branding
+    <t>Step-input-rettelser specifikation; FAQ-promotion-design</t>
+  </si>
+  <si>
+    <t>Sidste fulde arbejdsuge før sommer.</t>
+  </si>
+  <si>
+    <t>TS3 kreativt brief + sommer-forberedelse</t>
+  </si>
+  <si>
+    <t>• Brief TS3 kreativ til fotograf/freelance designer: lifestyle-billeder, kvinder 50+ i danske arbejds- og hjemmekontekster, vertikale mobil-først-formater, Hjerteforeningen co-branding
 • Brief omfatter: 3-4 helte-billeder, 6-8 social-kort, e-mail-overskrifter, betalt Meta-varianter
 • Klargør sommer-vedligeholdelsesliste</t>
   </si>
   <si>
-    <t xml:space="preserve">Hjerteforeningen logo-lockup skal godkendes af kampagneleder først.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sommer uge 1 — kun vedligehold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Overvåg Clarity for fejl
+    <t>Hjerteforeningen logo-lockup skal godkendes af kampagneleder først.</t>
+  </si>
+  <si>
+    <t>Sommer uge 1 — kun vedligehold</t>
+  </si>
+  <si>
+    <t>• Overvåg Clarity for fejl
 • Triage indkommende bug-rapporter
 • Gennemgå platform smart event-data — første 6 uger med tracking
 • Ingen nye design-opgaver</t>
   </si>
   <si>
-    <t xml:space="preserve">Smart events valideringsrapport</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stort set alle arbejdspladser på ferie. Let hånd.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sommer uge 2 — kun vedligehold</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Fortsæt overvågning
+    <t>Smart events valideringsrapport</t>
+  </si>
+  <si>
+    <t>Stort set alle arbejdspladser på ferie. Let hånd.</t>
+  </si>
+  <si>
+    <t>Sommer uge 2 — kun vedligehold</t>
+  </si>
+  <si>
+    <t>• Fortsæt overvågning
 • Dokumentér uventede mønstre til opfølgning efter sommer</t>
   </si>
   <si>
-    <t xml:space="preserve">Stille uge. Brug til personlig genopladning.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sommer uge 3 — LinkedIn-gennemgang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Gennemgang af LinkedIn-kampagne Clarity-data: engagerede landingssiden? Hvor faldt de fra?
+    <t>Stille uge. Brug til personlig genopladning.</t>
+  </si>
+  <si>
+    <t>Sommer uge 3 — LinkedIn-gennemgang</t>
+  </si>
+  <si>
+    <t>• Gennemgang af LinkedIn-kampagne Clarity-data: engagerede landingssiden? Hvor faldt de fra?
 • Tjek ind med TS3 kreativ produktion — leverancer skyldes uge 10
 • Let designarbejde på Hjerteforeningen-partnerskabs-side hvis nødvendigt</t>
   </si>
   <si>
-    <t xml:space="preserve">LinkedIn UX-gennemgang; kreativ checkpoint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sidste sommer-uge. Aktivitet ramper op herfra.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kreativ ankommer + platform-QA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Modtag TS3 kreative leverancer — gennemgå, giv feedback, færdiggør
+    <t>LinkedIn UX-gennemgang; kreativ checkpoint</t>
+  </si>
+  <si>
+    <t>Sidste sommer-uge. Aktivitet ramper op herfra.</t>
+  </si>
+  <si>
+    <t>Kreativ ankommer + platform-QA</t>
+  </si>
+  <si>
+    <t>• Modtag TS3 kreative leverancer — gennemgå, giv feedback, færdiggør
 • Påbegynd ende-til-ende QA på tilmeldingsflow: deltager, holdkaptajn, SammenholdsID-admin-stier
 • Test på Edge desktop, iOS Safari, Chrome Mobile
 • Endelig Hjerteforeningen co-branding-placering tjekket på tværs af site</t>
   </si>
   <si>
-    <t xml:space="preserve">Godkendt kreativ-bank; QA-runde 1 rapport</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase 3 starter midt på ugen. Arbejdet komprimeres herfra.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sidste platform-rettelser; QA-runde 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Lancér step-input-rettelser hvis QA er ren — koordinér med IT Heroes
+    <t>Godkendt kreativ-bank; QA-runde 1 rapport</t>
+  </si>
+  <si>
+    <t>Fase 3 starter midt på ugen. Arbejdet komprimeres herfra.</t>
+  </si>
+  <si>
+    <t>Sidste platform-rettelser; QA-runde 2</t>
+  </si>
+  <si>
+    <t>• Lancér step-input-rettelser hvis QA er ren — koordinér med IT Heroes
 • Anden QA-runde: fokus på edge cases og mobile flow
 • Verificér at Clarity smart events stadig fyrer efter deploys
 • Ret eventuelle blokerende fejl</t>
   </si>
   <si>
-    <t xml:space="preserve">Step-input-rettelser live (hvis ren); QA-runde 2 rapport</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sidste uge til at lancere UX-ændringer. Alt der ikke er klart fredag udskydes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Freeze-forberedelse + lancerings-klargøring</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Endelig QA på alle kritiske stier
+    <t>Step-input-rettelser live (hvis ren); QA-runde 2 rapport</t>
+  </si>
+  <si>
+    <t>Sidste uge til at lancere UX-ændringer. Alt der ikke er klart fredag udskydes.</t>
+  </si>
+  <si>
+    <t>Freeze-forberedelse + lancerings-klargøring</t>
+  </si>
+  <si>
+    <t>• Endelig QA på alle kritiske stier
 • Site + platform freeze annonceret til mandag 24. aug
 • Dokumentér kendte problemer til IT Heroes-overvågning
 • Bekræft Clarity, smart events, alt fyrer</t>
   </si>
   <si>
-    <t xml:space="preserve">Freeze-tjekliste godkendt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ingen nye design-opgaver denne uge. Kun stabilisering.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sidste uge før TS3 live</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Freeze i kraft: ingen risikable deploys
+    <t>Freeze-tjekliste godkendt</t>
+  </si>
+  <si>
+    <t>Ingen nye design-opgaver denne uge. Kun stabilisering.</t>
+  </si>
+  <si>
+    <t>Sidste uge før TS3 live</t>
+  </si>
+  <si>
+    <t>• Freeze i kraft: ingen risikable deploys
 • Endelig røg-test fredag
 • Klargør daglig overvågnings-dashboard til kampagne-launch
 • Stå standby til mandag morgen go-live</t>
   </si>
   <si>
-    <t xml:space="preserve">Daglig overvågnings-dashboard klar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holdkaptajner tilmelder denne uge. Hold øje med friktion i realtid.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS3 live — uge 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Daglig Clarity-gennemgang (15-30 min): step-input, statistik, profilside
+    <t>Daglig overvågnings-dashboard klar</t>
+  </si>
+  <si>
+    <t>Holdkaptajner tilmelder denne uge. Hold øje med friktion i realtid.</t>
+  </si>
+  <si>
+    <t>TS3 live — uge 1</t>
+  </si>
+  <si>
+    <t>• Daglig Clarity-gennemgang (15-30 min): step-input, statistik, profilside
 • Smart events overvågning: tilmeldings-rate, første-skridt-rate
 • Daglig bug-triage med IT Heroes
 • Kun hotfixes — ingen nye funktioner</t>
   </si>
   <si>
-    <t xml:space="preserve">Daglige Clarity-noter; bug-triage log</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Højeste trafik-uge. Ting går i stykker. Vær tilgængelig.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS3 live — uge 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Fortsæt daglig overvågning
+    <t>Daglige Clarity-noter; bug-triage log</t>
+  </si>
+  <si>
+    <t>Højeste trafik-uge. Ting går i stykker. Vær tilgængelig.</t>
+  </si>
+  <si>
+    <t>TS3 live — uge 2</t>
+  </si>
+  <si>
+    <t>• Fortsæt daglig overvågning
 • Påbegynd efter-kampagne retrospektiv: hvad virkede, hvad gik i stykker, hvad skal rettes før TS4
 • Notér mønstre til mellem-kampagne-læring
 • Saml Walk of Fame-historier indsendt under kampagnen</t>
   </si>
   <si>
-    <t xml:space="preserve">Midt-kampagne retro-udkast påbegyndt; Walk of Fame-indsamling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kampagne slutter søndag 13. sep.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Efter-kampagne retrospektiv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Fuld Clarity-gennemgang af TS3 platform-data: sammenlign med TS3 2025 baseline
+    <t>Midt-kampagne retro-udkast påbegyndt; Walk of Fame-indsamling</t>
+  </si>
+  <si>
+    <t>Kampagne slutter søndag 13. sep.</t>
+  </si>
+  <si>
+    <t>Efter-kampagne retrospektiv</t>
+  </si>
+  <si>
+    <t>• Fuld Clarity-gennemgang af TS3 platform-data: sammenlign med TS3 2025 baseline
 • Forbedrede step-input-friktion? Faldt profilside-quickback-rate?
 • TS3 retrospektiv med IT Heroes: hvad gik i stykker, hvad virkede, hvad skal rettes før TS4
 • Dokumentér UX-læringer til næste kampagne-cyklus
 • Påbegynd scoping af TS4 (9-22. november)</t>
   </si>
   <si>
-    <t xml:space="preserve">TS3 UX-retro-dokument; TS4 scoping-noter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stille uge — brug til dyb retrospektiv. Næste kampagne er kun 8 uger væk.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marketingplan — TS3 2026 (Tæl Skridt For Hjertet × Hjerteforeningen)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mål: fastholde tidligere holdkaptajner (primært) + rekruttere nye arbejdspladser. Budget: 30.000 kr.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Målgruppe: danske kvinder 45+ på arbejdspladser (Edge, mandage 06-13). Holdkaptajn ofte HR/kommunikation/trivsel, 35-54.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kampagne-idéer forankret i Hjerteforeningen-partnerskabet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Idé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Beskrivelse</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hver 2. dansker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hjerteforeningens datapoint — hver anden dansker rammes af hjertesygdom — bruges som hovedkrog. Visuelt: 50% af et arbejdspladsfoto i sort/hvid, 50% i TS-orange. Caption: 'Hver anden af jer får en hjertesygdom. Tæl Skridt For Hjertet — fordi alle skridt beskytter hjertet.' Bruges på Meta, LinkedIn, e-mail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pulsér hverdagen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lånt fra partnerskabsteksten ('får hverdagen til at pulsere'). Kort video eller karrusel der viser, hvordan 10.000 skridt om dagen ser ud i en dansk arbejdsdag — kaffe på vej til møde, frokostgåtur, tur til kollegaen i stedet for Teams-besked. Hjerteforeningen-anker til sidst: 'Sådan passer vi på hjertet.'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holdkaptajn-tilbagekomst</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Målrettet e-mail + LinkedIn-annonce til tidligere holdkaptajner fra listen. Emnelinje: 'Dit hold venter — TS3 starter 31. august, og denne gang er det for hjertet.' Personlig, anerkender at de allerede har gjort arbejdet, lav barriere: bare klik 'kom tilbage'.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sundhed på arbejdspladsen — HR-vinklen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B2B-vinkel for SammenholdsID. Langt LinkedIn-opslag + e-mail: forebyggelse på arbejdspladsen er billigere end reaktiv sundhedsforsikring. Hjerteforeningen-partnerskabet giver troværdighed. Målrettet HR/kommunikation/trivsel-roller.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Det første skridt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Onboarding-fokuseret indhold til nye arbejdspladser: kort how-to-serie (tilmelding → første hold → første lod). Hostet på sitet, distribueret via betalt søgning og organisk social. Fjerner 'jeg forstår ikke, hvordan det virker'-barrieren.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Walk of Fame for hjertet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Under kampagnen: spotlight hold der går i mindet om nogen med hjertesygdom, eller af forebyggende årsager. Personligt, følelsesladet, passer til partnerskabet. Indsendelses-formular på sitet.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DR / nyhedspitch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kombinationen af Hjerteforeningens troværdighed + 48.000 deltagere + hjertesundheds-vinkel er pitchbar til danske nyhedsdesks (sundhed, livsstil, erhverv). Værd at lave et fokuseret PR-push i fase 3, selv uden budget — bare en velskrevet e-mail til 5-10 relevante journalister.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ugentlig marketing-plan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aktive kanaler</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Opgaver / udsendelser</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Budget denne uge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail, organisk social</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Indfør nye UTM-konventioner på tværs af alle kanaler (utm_campaign=ts3-2026-prelaunch osv.)
+    <t>TS3 UX-retro-dokument; TS4 scoping-noter</t>
+  </si>
+  <si>
+    <t>Stille uge — brug til dyb retrospektiv. Næste kampagne er kun 8 uger væk.</t>
+  </si>
+  <si>
+    <t>Marketingplan — TS3 2026 (Tæl Skridt For Hjertet × Hjerteforeningen)</t>
+  </si>
+  <si>
+    <t>Mål: fastholde tidligere holdkaptajner (primært) + rekruttere nye arbejdspladser. Budget: 30.000 kr.</t>
+  </si>
+  <si>
+    <t>Målgruppe: danske kvinder 45+ på arbejdspladser (Edge, mandage 06-13). Holdkaptajn ofte HR/kommunikation/trivsel, 35-54.</t>
+  </si>
+  <si>
+    <t>Kampagne-idéer forankret i Hjerteforeningen-partnerskabet</t>
+  </si>
+  <si>
+    <t>Idé</t>
+  </si>
+  <si>
+    <t>Beskrivelse</t>
+  </si>
+  <si>
+    <t>Hver 2. dansker</t>
+  </si>
+  <si>
+    <t>Hjerteforeningens datapoint — hver anden dansker rammes af hjertesygdom — bruges som hovedkrog. Visuelt: 50% af et arbejdspladsfoto i sort/hvid, 50% i TS-orange. Caption: 'Hver anden af jer får en hjertesygdom. Tæl Skridt For Hjertet — fordi alle skridt beskytter hjertet.' Bruges på Meta, LinkedIn, e-mail.</t>
+  </si>
+  <si>
+    <t>Pulsér hverdagen</t>
+  </si>
+  <si>
+    <t>Lånt fra partnerskabsteksten ('får hverdagen til at pulsere'). Kort video eller karrusel der viser, hvordan 10.000 skridt om dagen ser ud i en dansk arbejdsdag — kaffe på vej til møde, frokostgåtur, tur til kollegaen i stedet for Teams-besked. Hjerteforeningen-anker til sidst: 'Sådan passer vi på hjertet.'</t>
+  </si>
+  <si>
+    <t>Holdkaptajn-tilbagekomst</t>
+  </si>
+  <si>
+    <t>Målrettet e-mail + LinkedIn-annonce til tidligere holdkaptajner fra listen. Emnelinje: 'Dit hold venter — TS3 starter 31. august, og denne gang er det for hjertet.' Personlig, anerkender at de allerede har gjort arbejdet, lav barriere: bare klik 'kom tilbage'.</t>
+  </si>
+  <si>
+    <t>Sundhed på arbejdspladsen — HR-vinklen</t>
+  </si>
+  <si>
+    <t>B2B-vinkel for SammenholdsID. Langt LinkedIn-opslag + e-mail: forebyggelse på arbejdspladsen er billigere end reaktiv sundhedsforsikring. Hjerteforeningen-partnerskabet giver troværdighed. Målrettet HR/kommunikation/trivsel-roller.</t>
+  </si>
+  <si>
+    <t>Det første skridt</t>
+  </si>
+  <si>
+    <t>Onboarding-fokuseret indhold til nye arbejdspladser: kort how-to-serie (tilmelding → første hold → første lod). Hostet på sitet, distribueret via betalt søgning og organisk social. Fjerner 'jeg forstår ikke, hvordan det virker'-barrieren.</t>
+  </si>
+  <si>
+    <t>Walk of Fame for hjertet</t>
+  </si>
+  <si>
+    <t>Under kampagnen: spotlight hold der går i mindet om nogen med hjertesygdom, eller af forebyggende årsager. Personligt, følelsesladet, passer til partnerskabet. Indsendelses-formular på sitet.</t>
+  </si>
+  <si>
+    <t>DR / nyhedspitch</t>
+  </si>
+  <si>
+    <t>Kombinationen af Hjerteforeningens troværdighed + 48.000 deltagere + hjertesundheds-vinkel er pitchbar til danske nyhedsdesks (sundhed, livsstil, erhverv). Værd at lave et fokuseret PR-push i fase 3, selv uden budget — bare en velskrevet e-mail til 5-10 relevante journalister.</t>
+  </si>
+  <si>
+    <t>Ugentlig marketing-plan</t>
+  </si>
+  <si>
+    <t>Aktive kanaler</t>
+  </si>
+  <si>
+    <t>Opgaver / udsendelser</t>
+  </si>
+  <si>
+    <t>Budget denne uge</t>
+  </si>
+  <si>
+    <t>E-mail, organisk social</t>
+  </si>
+  <si>
+    <t>• Indfør nye UTM-konventioner på tværs af alle kanaler (utm_campaign=ts3-2026-prelaunch osv.)
 • Brief LinkedIn-test kreativ — SammenholdsID-fokuseret, B2B-vinkel
 • Opsæt LinkedIn-annoncekonto hvis ikke gjort
 • E-mail til tidligere holdkaptajner: 'Save the date: TS3 starter 31. august — denne gang med Hjerteforeningen'
 • Organisk Facebook-opslag: dato-annoncering med Hjerteforeningen-logo</t>
   </si>
   <si>
-    <t xml:space="preserve">0 kr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UTM-oprydning er den vigtigste rettelse denne uge.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LinkedIn-test live</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail, organisk social, LinkedIn betalt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Lancér LinkedIn-annoncesæt: SammenholdsID, målret HR/kommunikation/trivsel i danske arbejdspladser 50+ ansatte (~7.000 kr / 4 uger)
+    <t>0 kr</t>
+  </si>
+  <si>
+    <t>UTM-oprydning er den vigtigste rettelse denne uge.</t>
+  </si>
+  <si>
+    <t>LinkedIn-test live</t>
+  </si>
+  <si>
+    <t>E-mail, organisk social, LinkedIn betalt</t>
+  </si>
+  <si>
+    <t>• Lancér LinkedIn-annoncesæt: SammenholdsID, målret HR/kommunikation/trivsel i danske arbejdspladser 50+ ansatte (~7.000 kr / 4 uger)
 • Første Walk of Fame-historie (organisk Facebook + LinkedIn)
 • Nyhedsbrev-tilmelding fremhævet på nyt forside-design
 • E-mail-udsendelse: 'Hver 2. dansker'-kampagneidé — etablerer partnerskabshistorien</t>
   </si>
   <si>
-    <t xml:space="preserve">1.750 kr (LinkedIn uge 1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mandag morgen-udsendelse for e-mail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Listebygning + Hjerteforeningen-historie</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Langt opslag: 'Hvorfor Tæl Skridt og Hjerteforeningen?' — publiceret på TS-site, delt på LinkedIn og Facebook
+    <t>1.750 kr (LinkedIn uge 1)</t>
+  </si>
+  <si>
+    <t>Mandag morgen-udsendelse for e-mail.</t>
+  </si>
+  <si>
+    <t>Listebygning + Hjerteforeningen-historie</t>
+  </si>
+  <si>
+    <t>• Langt opslag: 'Hvorfor Tæl Skridt og Hjerteforeningen?' — publiceret på TS-site, delt på LinkedIn og Facebook
 • Anden Walk of Fame-historie
 • Boost nyhedsbrev-tilmelding ('Få besked')
 • LinkedIn-annonce fortsætter</t>
   </si>
   <si>
-    <t xml:space="preserve">1.750 kr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Langt indhold virker for denne målgruppe (50% nyhedslæsere).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holdkaptajn-fastholdelses-push</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Målrettet e-mail til tidligere holdkaptajner: 'Holdkaptajn-tilbagekomst'-kampagne — personlig, lav-friktion CTA
+    <t>1.750 kr</t>
+  </si>
+  <si>
+    <t>Langt indhold virker for denne målgruppe (50% nyhedslæsere).</t>
+  </si>
+  <si>
+    <t>Holdkaptajn-fastholdelses-push</t>
+  </si>
+  <si>
+    <t>• Målrettet e-mail til tidligere holdkaptajner: 'Holdkaptajn-tilbagekomst'-kampagne — personlig, lav-friktion CTA
 • Segmentér listen: tidligere holdkaptajner der IKKE allerede har tilmeldt TS3
 • Tredje Walk of Fame-historie
 • LinkedIn-annonce uge 3</t>
   </si>
   <si>
-    <t xml:space="preserve">Vigtigste e-mail i fase 1. A/B-test emnelinjer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hjerteforeningen formel annoncering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Formel partnerskabs-annonceringsopslag — co-brandet, med begge logoer, statement fra begge parter
+    <t>Vigtigste e-mail i fase 1. A/B-test emnelinjer.</t>
+  </si>
+  <si>
+    <t>Hjerteforeningen formel annoncering</t>
+  </si>
+  <si>
+    <t>• Formel partnerskabs-annonceringsopslag — co-brandet, med begge logoer, statement fra begge parter
 • E-mail til hele listen med partnerskabshistorien
 • LinkedIn-annonce sidste uge
 • Før-sommer 'sidste push før sommerferien'-e-mail</t>
   </si>
   <si>
-    <t xml:space="preserve">1.750 kr (LinkedIn uge 4 slut)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slut på LinkedIn fase 1-test.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sidste uge før sommer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Før-sommer e-mail-blast: 'Vi tager en pause — vi ses i august. Husk: TS3 starter 31. august'
+    <t>1.750 kr (LinkedIn uge 4 slut)</t>
+  </si>
+  <si>
+    <t>Slut på LinkedIn fase 1-test.</t>
+  </si>
+  <si>
+    <t>Sidste uge før sommer</t>
+  </si>
+  <si>
+    <t>• Før-sommer e-mail-blast: 'Vi tager en pause — vi ses i august. Husk: TS3 starter 31. august'
 • 'Pulsér hverdagen'-video/karrusel går live på organisk
 • Saml LinkedIn fase 1-resultater, forbered beslutningsdokument</t>
   </si>
   <si>
-    <t xml:space="preserve">Sidste meningsfulde kommunikation før sommer-dødvande.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sommerpause</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kun organisk social (Benspænd)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• 1 organisk Facebook-opslag — Benspænd-fokuseret, lifestyle, lavmælt
+    <t>Sidste meningsfulde kommunikation før sommer-dødvande.</t>
+  </si>
+  <si>
+    <t>Sommerpause</t>
+  </si>
+  <si>
+    <t>Kun organisk social (Benspænd)</t>
+  </si>
+  <si>
+    <t>• 1 organisk Facebook-opslag — Benspænd-fokuseret, lifestyle, lavmælt
 • Ingen betalt, ingen e-mail
 • Nyhedsbrev-tilmelding forbliver live på sitet</t>
   </si>
   <si>
-    <t xml:space="preserve">Arbejdspladser lukkede.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kun organisk social</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• 1 organisk Facebook-opslag — Walk of Fame eller Benspænd
+    <t>Arbejdspladser lukkede.</t>
+  </si>
+  <si>
+    <t>Kun organisk social</t>
+  </si>
+  <si>
+    <t>• 1 organisk Facebook-opslag — Walk of Fame eller Benspænd
 • Vedligehold nyhedsbrev-tilmelding
 • Planlæg/forbered august-relancering</t>
   </si>
   <si>
-    <t xml:space="preserve">Stille uge.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sommer-slut + LinkedIn-beslutning</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Organisk social</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• 1 organisk opslag der antyder TS3 — 'En måned til. Er du klar?'
+    <t>Stille uge.</t>
+  </si>
+  <si>
+    <t>Sommer-slut + LinkedIn-beslutning</t>
+  </si>
+  <si>
+    <t>Organisk social</t>
+  </si>
+  <si>
+    <t>• 1 organisk opslag der antyder TS3 — 'En måned til. Er du klar?'
 • Færdiggør LinkedIn-skalerings-beslutning baseret på fase 1-resultater
 • Brief eventuelle yderligere betalte Meta-kreativer
 • Verificér kreativ-leverancer skyldes uge 10</t>
   </si>
   <si>
-    <t xml:space="preserve">Vækkelses-signal-uge. Blødt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase 3 optakt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail, organisk social, betalt Meta soft-start</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• E-mail: 'Vi er tilbage — TS3 starter om 4 uger'
+    <t>Vækkelses-signal-uge. Blødt.</t>
+  </si>
+  <si>
+    <t>Fase 3 optakt</t>
+  </si>
+  <si>
+    <t>E-mail, organisk social, betalt Meta soft-start</t>
+  </si>
+  <si>
+    <t>• E-mail: 'Vi er tilbage — TS3 starter om 4 uger'
 • Begynd betalt Meta soft-launch (lavt budget, bred målretning) — test kreativ-varianter
 • Daglige organiske opslag: nedtælling begynder
 • 'Det første skridt'-onboarding-indhold går live på sitet</t>
   </si>
   <si>
-    <t xml:space="preserve">1.500 kr (Meta soft)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fase 3 starter midt på ugen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aktiv rekruttering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail, organisk social, betalt Meta, betalt Google, LinkedIn (hvis skaleret)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Betalt Meta skaleret til fuldt budget (~4.000 kr denne uge)
+    <t>1.500 kr (Meta soft)</t>
+  </si>
+  <si>
+    <t>Fase 3 starter midt på ugen.</t>
+  </si>
+  <si>
+    <t>Aktiv rekruttering</t>
+  </si>
+  <si>
+    <t>E-mail, organisk social, betalt Meta, betalt Google, LinkedIn (hvis skaleret)</t>
+  </si>
+  <si>
+    <t>• Betalt Meta skaleret til fuldt budget (~4.000 kr denne uge)
 • Betalt Google Search lanceres: brandede + kategori-relaterede søgeord (~1.500 kr denne uge)
 • LinkedIn-skalering hvis godkendt (~1.500 kr)
 • E-mail: 'Sundhed på arbejdspladsen'-vinkel til HR/SammenholdsID-liste
 • 2-3 organiske opslag: variationer af 'Hver 2. dansker'-kreativ</t>
   </si>
   <si>
-    <t xml:space="preserve">Højeste ugentlige spend indtil kampagne live.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sidste uge før lancering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail, organisk social, betalt Meta, betalt Google, LinkedIn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• E-mail-blast til hele listen: 'TS3 starter på mandag. Sidste chance for at melde sig til'
+    <t>Højeste ugentlige spend indtil kampagne live.</t>
+  </si>
+  <si>
+    <t>Sidste uge før lancering</t>
+  </si>
+  <si>
+    <t>E-mail, organisk social, betalt Meta, betalt Google, LinkedIn</t>
+  </si>
+  <si>
+    <t>• E-mail-blast til hele listen: 'TS3 starter på mandag. Sidste chance for at melde sig til'
 • Betalt Meta fortsætter (~4.000 kr)
 • Betalt Google fortsætter (~1.500 kr)
 • LinkedIn final-push hvis kører
 • PR-push: pitch til danske nyhedsdesks (sundhed, livsstil, erhverv) — 5-10 journalister, velskrevet e-mail</t>
   </si>
   <si>
-    <t xml:space="preserve">6.500 kr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sidste uge med aktiv rekruttering.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lanceringsuge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail, organisk social, betalt Meta, betalt Google</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sidste-chance-e-mail: 'TS3 begynder på søndag — sidste chance'
+    <t>6.500 kr</t>
+  </si>
+  <si>
+    <t>Sidste uge med aktiv rekruttering.</t>
+  </si>
+  <si>
+    <t>Lanceringsuge</t>
+  </si>
+  <si>
+    <t>E-mail, organisk social, betalt Meta, betalt Google</t>
+  </si>
+  <si>
+    <t>• Sidste-chance-e-mail: 'TS3 begynder på søndag — sidste chance'
 • Betalt Meta og Google trappes ned efterhånden som tilmelding lukker
 • Organisk nedtælling intensiveres: fredag-opslag, søndag-aften-opslag
 • Send 'Walk of Fame for hjertet'-indsendelses-formular til tidligere Walk of Fame-deltagere</t>
   </si>
   <si>
-    <t xml:space="preserve">3.500 kr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">De fleste arbejdspladser har commited inden onsdag.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kampagne live — uge 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-mail, organisk social (daglig)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Mandag: kampagne-kickoff-opslag (organisk Facebook + LinkedIn + Instagram)
+    <t>3.500 kr</t>
+  </si>
+  <si>
+    <t>De fleste arbejdspladser har commited inden onsdag.</t>
+  </si>
+  <si>
+    <t>Kampagne live — uge 1</t>
+  </si>
+  <si>
+    <t>E-mail, organisk social (daglig)</t>
+  </si>
+  <si>
+    <t>• Mandag: kampagne-kickoff-opslag (organisk Facebook + LinkedIn + Instagram)
 • Tirsdag e-mail: 'I gang — sådan kommer du godt fra start' (deltager-fokuseret)
 • Daglige organiske opslag: lykkehjul-vindere, holdkaptajn-shout-outs, Hjerteforeningen-hjertesundheds-tips
 • Stop alt betalt — skift til engagement</t>
   </si>
   <si>
-    <t xml:space="preserve">Marketing-fokus skifter til fastholdelse/engagement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kampagne live — uge 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Midt-uges e-mail: 'Hold momentum — du er halvvejs' (motivation + resterende lodder-matematik)
+    <t>Marketing-fokus skifter til fastholdelse/engagement.</t>
+  </si>
+  <si>
+    <t>Kampagne live — uge 2</t>
+  </si>
+  <si>
+    <t>• Midt-uges e-mail: 'Hold momentum — du er halvvejs' (motivation + resterende lodder-matematik)
 • Daglig organisk: topholds-spotlight, Walk of Fame for hjertet-indsendelser, Hjerteforeningen-indhold
 • Fredag e-mail: 'Sidste weekend — gør det tæller'
 • Søndag aften: tak-opslag; kampagne slutter</t>
   </si>
   <si>
-    <t xml:space="preserve">Sidste kampagne-uge. Planlæg efter-kampagne-retro til uge 38.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Mandag: tak-e-mail til alle deltagere — vinder-annoncering, Walk of Fame-højdepunkter
+    <t>Sidste kampagne-uge. Planlæg efter-kampagne-retro til uge 38.</t>
+  </si>
+  <si>
+    <t>• Mandag: tak-e-mail til alle deltagere — vinder-annoncering, Walk of Fame-højdepunkter
 • Midt-uges opslag: resultats-opsummering med Hjerteforeningen co-branding
 • Send Walk of Fame indsendelses-deadline-påmindelse
 • Saml marketing-retrospektiv: kanal-for-kanal performance, hvad skal gentages til TS4, hvad skal droppes</t>
   </si>
   <si>
-    <t xml:space="preserve">Stille uge til spend. Brug til dyb analyse — TS4 starter 9. november.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SAMLET BUDGET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimat baseret på ugentlige tal ovenfor:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">≈ 30.000 kr</t>
+    <t>Stille uge til spend. Brug til dyb analyse — TS4 starter 9. november.</t>
+  </si>
+  <si>
+    <t>SAMLET BUDGET</t>
+  </si>
+  <si>
+    <t>Estimat baseret på ugentlige tal ovenfor:</t>
+  </si>
+  <si>
+    <t>≈ 30.000 kr</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="17">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1045,115 +1047,87 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="18"/>
       <color rgb="FF16293E"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="10"/>
       <color rgb="FF9E9E9E"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF16293E"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="9"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="12"/>
       <color rgb="FF16293E"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <color rgb="FFEC9535"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="10"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FFEC9535"/>
       <name val="Calibri"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -1202,14 +1176,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin">
         <color rgb="FFD0D0D0"/>
       </left>
@@ -1225,297 +1199,174 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="64">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1574,47 +1425,63 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF16293E"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -1622,12 +1489,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -1656,7 +1523,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1677,7 +1544,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1728,7 +1595,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1746,51 +1613,50 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F47"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="32"/>
+    <col min="1" max="1" width="54.44140625" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="38" customWidth="1"/>
+    <col min="5" max="5" width="42" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:3" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:3" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
@@ -1798,7 +1664,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:3" ht="69" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>6</v>
       </c>
@@ -1806,7 +1672,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:3" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>8</v>
       </c>
@@ -1814,7 +1680,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:3" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>10</v>
       </c>
@@ -1822,7 +1688,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:3" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>12</v>
       </c>
@@ -1830,12 +1696,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
         <v>15</v>
       </c>
@@ -1846,7 +1712,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
         <v>18</v>
       </c>
@@ -1857,7 +1723,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:3" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
         <v>21</v>
       </c>
@@ -1868,7 +1734,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:3" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A16" s="11" t="s">
         <v>24</v>
       </c>
@@ -1879,7 +1745,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>27</v>
       </c>
@@ -1890,7 +1756,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A18" s="11" t="s">
         <v>30</v>
       </c>
@@ -1901,7 +1767,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>33</v>
       </c>
@@ -1912,12 +1778,12 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
         <v>37</v>
       </c>
@@ -1928,7 +1794,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A23" s="13" t="s">
         <v>40</v>
       </c>
@@ -1939,7 +1805,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A24" s="13" t="s">
         <v>43</v>
       </c>
@@ -1950,7 +1816,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:6" ht="55.2" x14ac:dyDescent="0.3">
       <c r="A25" s="13" t="s">
         <v>46</v>
       </c>
@@ -1961,7 +1827,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A26" s="13" t="s">
         <v>49</v>
       </c>
@@ -1972,7 +1838,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A27" s="13" t="s">
         <v>52</v>
       </c>
@@ -1983,7 +1849,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:6" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A28" s="13" t="s">
         <v>55</v>
       </c>
@@ -1994,12 +1860,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="14" t="s">
         <v>59</v>
       </c>
@@ -2019,7 +1885,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="15" t="s">
         <v>65</v>
       </c>
@@ -2039,7 +1905,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="15" t="s">
         <v>71</v>
       </c>
@@ -2059,7 +1925,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="15" t="s">
         <v>76</v>
       </c>
@@ -2079,7 +1945,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="15" t="s">
         <v>81</v>
       </c>
@@ -2099,7 +1965,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="15" t="s">
         <v>86</v>
       </c>
@@ -2119,7 +1985,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="19" t="s">
         <v>91</v>
       </c>
@@ -2139,7 +2005,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="19" t="s">
         <v>97</v>
       </c>
@@ -2159,7 +2025,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="19" t="s">
         <v>102</v>
       </c>
@@ -2179,7 +2045,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="19" t="s">
         <v>105</v>
       </c>
@@ -2199,7 +2065,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="19" t="s">
         <v>110</v>
       </c>
@@ -2219,7 +2085,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="42" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="22" t="s">
         <v>115</v>
       </c>
@@ -2239,7 +2105,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="22" t="s">
         <v>121</v>
       </c>
@@ -2259,7 +2125,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="22" t="s">
         <v>126</v>
       </c>
@@ -2279,7 +2145,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="26" t="s">
         <v>131</v>
       </c>
@@ -2299,7 +2165,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="26" t="s">
         <v>137</v>
       </c>
@@ -2319,7 +2185,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" spans="1:6" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="30" t="s">
         <v>142</v>
       </c>
@@ -2340,44 +2206,36 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G20"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="28"/>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:7" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="14" t="s">
         <v>59</v>
       </c>
@@ -2400,7 +2258,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:7" ht="87" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="34" t="s">
         <v>65</v>
       </c>
@@ -2423,7 +2281,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:7" ht="84" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="34" t="s">
         <v>71</v>
       </c>
@@ -2446,7 +2304,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:7" ht="87.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="34" t="s">
         <v>76</v>
       </c>
@@ -2469,7 +2327,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:7" ht="75.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="34" t="s">
         <v>81</v>
       </c>
@@ -2492,7 +2350,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:7" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="34" t="s">
         <v>86</v>
       </c>
@@ -2515,7 +2373,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:7" ht="93.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="38" t="s">
         <v>91</v>
       </c>
@@ -2538,7 +2396,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:7" ht="73.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="38" t="s">
         <v>97</v>
       </c>
@@ -2561,7 +2419,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="38" t="s">
         <v>102</v>
       </c>
@@ -2584,7 +2442,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:7" ht="87" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="38" t="s">
         <v>105</v>
       </c>
@@ -2607,7 +2465,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:7" ht="101.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="38" t="s">
         <v>110</v>
       </c>
@@ -2630,7 +2488,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:7" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="42" t="s">
         <v>115</v>
       </c>
@@ -2653,7 +2511,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="42" t="s">
         <v>121</v>
       </c>
@@ -2676,7 +2534,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:7" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="42" t="s">
         <v>126</v>
       </c>
@@ -2699,7 +2557,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:7" ht="87.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="46" t="s">
         <v>131</v>
       </c>
@@ -2722,7 +2580,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:7" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="46" t="s">
         <v>137</v>
       </c>
@@ -2745,7 +2603,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:7" ht="111.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="50" t="s">
         <v>142</v>
       </c>
@@ -2769,55 +2627,47 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H35"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="28"/>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="75.88671875" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
+    <col min="6" max="6" width="52" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:2" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="54" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>220</v>
       </c>
@@ -2825,7 +2675,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:2" ht="72.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="38" t="s">
         <v>222</v>
       </c>
@@ -2833,7 +2683,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:2" ht="79.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="38" t="s">
         <v>224</v>
       </c>
@@ -2841,7 +2691,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:2" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="38" t="s">
         <v>226</v>
       </c>
@@ -2849,7 +2699,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:2" ht="70.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="38" t="s">
         <v>228</v>
       </c>
@@ -2857,7 +2707,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:2" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="38" t="s">
         <v>230</v>
       </c>
@@ -2865,7 +2715,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="38" t="s">
         <v>232</v>
       </c>
@@ -2873,7 +2723,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="38" t="s">
         <v>234</v>
       </c>
@@ -2881,12 +2731,12 @@
         <v>235</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="54" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="14" t="s">
         <v>59</v>
       </c>
@@ -2912,7 +2762,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:8" ht="117.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="34" t="s">
         <v>65</v>
       </c>
@@ -2938,7 +2788,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:8" ht="108" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="34" t="s">
         <v>71</v>
       </c>
@@ -2964,7 +2814,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:8" ht="75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="34" t="s">
         <v>76</v>
       </c>
@@ -2990,7 +2840,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:8" ht="83.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="34" t="s">
         <v>81</v>
       </c>
@@ -3016,7 +2866,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:8" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="34" t="s">
         <v>86</v>
       </c>
@@ -3042,7 +2892,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:8" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="38" t="s">
         <v>91</v>
       </c>
@@ -3068,7 +2918,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:8" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="38" t="s">
         <v>97</v>
       </c>
@@ -3094,7 +2944,7 @@
         <v>266</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:8" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="38" t="s">
         <v>102</v>
       </c>
@@ -3120,7 +2970,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:8" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="38" t="s">
         <v>105</v>
       </c>
@@ -3146,7 +2996,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:8" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="38" t="s">
         <v>110</v>
       </c>
@@ -3172,7 +3022,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:8" ht="102" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="42" t="s">
         <v>115</v>
       </c>
@@ -3198,7 +3048,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:8" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="42" t="s">
         <v>121</v>
       </c>
@@ -3224,7 +3074,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="42" t="s">
         <v>126</v>
       </c>
@@ -3250,7 +3100,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:8" ht="97.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="46" t="s">
         <v>131</v>
       </c>
@@ -3276,7 +3126,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:8" ht="91.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="46" t="s">
         <v>137</v>
       </c>
@@ -3302,7 +3152,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="69.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:8" ht="99" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="50" t="s">
         <v>142</v>
       </c>
@@ -3328,7 +3178,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="60" t="s">
         <v>302</v>
       </c>
@@ -3345,12 +3195,7 @@
       <c r="H35" s="61"/>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>